<commit_message>
chore(data-release): publish site data 2026-10-23 02:01:21 UTC
</commit_message>
<xml_diff>
--- a/countries/au/2026-2029.xlsx
+++ b/countries/au/2026-2029.xlsx
@@ -66594,13 +66594,13 @@
         </is>
       </c>
       <c r="N480" t="n">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="O480" t="n">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="R480" t="n">
-        <v>1.597673141491109</v>
+        <v>1.594000329671589</v>
       </c>
       <c r="U480" t="inlineStr">
         <is>
@@ -67962,13 +67962,13 @@
         </is>
       </c>
       <c r="N490" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="O490" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="R490" t="n">
-        <v>0.4627742892594935</v>
+        <v>0.4591014774399738</v>
       </c>
       <c r="AA490" t="inlineStr">
         <is>
@@ -69600,13 +69600,13 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O502" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R502" t="n">
-        <v>0.01101843545855937</v>
+        <v>0.01469124727807916</v>
       </c>
       <c r="AA502" t="inlineStr">
         <is>
@@ -70703,13 +70703,13 @@
         </is>
       </c>
       <c r="N510" t="n">
-        <v>7515</v>
+        <v>7519</v>
       </c>
       <c r="O510" t="n">
-        <v>7515</v>
+        <v>7519</v>
       </c>
       <c r="R510" t="n">
-        <v>27.60118082369122</v>
+        <v>27.6158720709693</v>
       </c>
       <c r="AA510" t="inlineStr">
         <is>
@@ -71108,13 +71108,13 @@
         </is>
       </c>
       <c r="N513" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="O513" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="R513" t="n">
-        <v>0.8116914121138735</v>
+        <v>0.8153642239333934</v>
       </c>
       <c r="AA513" t="inlineStr">
         <is>
@@ -71378,13 +71378,13 @@
         </is>
       </c>
       <c r="N515" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="O515" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="R515" t="n">
-        <v>0.2130230855321478</v>
+        <v>0.2166958973516676</v>
       </c>
       <c r="AA515" t="inlineStr">
         <is>
@@ -71918,13 +71918,13 @@
         </is>
       </c>
       <c r="N519" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O519" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R519" t="n">
-        <v>0.2497512037273457</v>
+        <v>0.2534240155468655</v>
       </c>
       <c r="AA519" t="inlineStr">
         <is>
@@ -73133,13 +73133,13 @@
         </is>
       </c>
       <c r="N528" t="n">
-        <v>19124</v>
+        <v>19126</v>
       </c>
       <c r="O528" t="n">
-        <v>19124</v>
+        <v>19126</v>
       </c>
       <c r="R528" t="n">
-        <v>70.23885323649647</v>
+        <v>70.24619886013551</v>
       </c>
       <c r="AA528" t="inlineStr">
         <is>
@@ -73808,13 +73808,13 @@
         </is>
       </c>
       <c r="N533" t="n">
-        <v>3629</v>
+        <v>3614</v>
       </c>
       <c r="O533" t="n">
-        <v>3629</v>
+        <v>3614</v>
       </c>
       <c r="R533" t="n">
-        <v>13.32863409303732</v>
+        <v>13.27354191574452</v>
       </c>
       <c r="AA533" t="inlineStr">
         <is>
@@ -75626,13 +75626,13 @@
         </is>
       </c>
       <c r="N546" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O546" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="R546" t="n">
-        <v>1.002677626728903</v>
+        <v>1.006350438548423</v>
       </c>
       <c r="U546" t="inlineStr">
         <is>
@@ -76049,13 +76049,13 @@
         </is>
       </c>
       <c r="N549" t="n">
-        <v>7387</v>
+        <v>7388</v>
       </c>
       <c r="O549" t="n">
-        <v>7387</v>
+        <v>7388</v>
       </c>
       <c r="R549" t="n">
-        <v>27.13106091079269</v>
+        <v>27.13473372261221</v>
       </c>
       <c r="AA549" t="inlineStr">
         <is>
@@ -76319,13 +76319,13 @@
         </is>
       </c>
       <c r="N551" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O551" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R551" t="n">
-        <v>0.08814748366847497</v>
+        <v>0.09182029548799475</v>
       </c>
       <c r="AA551" t="inlineStr">
         <is>
@@ -76454,13 +76454,13 @@
         </is>
       </c>
       <c r="N552" t="n">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="O552" t="n">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="R552" t="n">
-        <v>1.531562528739753</v>
+        <v>1.524216905100713</v>
       </c>
       <c r="U552" t="inlineStr">
         <is>
@@ -76598,13 +76598,13 @@
         </is>
       </c>
       <c r="N553" t="n">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="O553" t="n">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="R553" t="n">
-        <v>1.777640920647578</v>
+        <v>1.773968108828059</v>
       </c>
       <c r="U553" t="inlineStr">
         <is>
@@ -76877,13 +76877,13 @@
         </is>
       </c>
       <c r="N555" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O555" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R555" t="n">
-        <v>0</v>
+        <v>0.00367281181951979</v>
       </c>
       <c r="AA555" t="inlineStr">
         <is>
@@ -77552,13 +77552,13 @@
         </is>
       </c>
       <c r="N560" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O560" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="R560" t="n">
-        <v>0.209350273712628</v>
+        <v>0.2056774618931082</v>
       </c>
       <c r="AA560" t="inlineStr">
         <is>
@@ -78776,13 +78776,13 @@
         </is>
       </c>
       <c r="N569" t="n">
-        <v>71102</v>
+        <v>71104</v>
       </c>
       <c r="O569" t="n">
-        <v>71102</v>
+        <v>71104</v>
       </c>
       <c r="R569" t="n">
-        <v>261.1442659914961</v>
+        <v>261.1516116151352</v>
       </c>
       <c r="AA569" t="inlineStr">
         <is>
@@ -78911,13 +78911,13 @@
         </is>
       </c>
       <c r="N570" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O570" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R570" t="n">
-        <v>0.02938249455615832</v>
+        <v>0.03305530637567811</v>
       </c>
       <c r="AA570" t="inlineStr">
         <is>
@@ -79460,13 +79460,13 @@
         </is>
       </c>
       <c r="N574" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O574" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R574" t="n">
-        <v>0.00367281181951979</v>
+        <v>0</v>
       </c>
       <c r="AA574" t="inlineStr">
         <is>
@@ -79735,13 +79735,13 @@
         </is>
       </c>
       <c r="N576" t="n">
-        <v>886</v>
+        <v>889</v>
       </c>
       <c r="O576" t="n">
-        <v>886</v>
+        <v>889</v>
       </c>
       <c r="R576" t="n">
-        <v>3.254111272094534</v>
+        <v>3.265129707553093</v>
       </c>
       <c r="U576" t="inlineStr">
         <is>
@@ -79879,13 +79879,13 @@
         </is>
       </c>
       <c r="N577" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O577" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R577" t="n">
-        <v>0.1358940373222322</v>
+        <v>0.139566849141752</v>
       </c>
       <c r="AA577" t="inlineStr">
         <is>
@@ -80563,13 +80563,13 @@
         </is>
       </c>
       <c r="N582" t="n">
-        <v>7518</v>
+        <v>7525</v>
       </c>
       <c r="O582" t="n">
-        <v>7518</v>
+        <v>7525</v>
       </c>
       <c r="R582" t="n">
-        <v>27.61219925914978</v>
+        <v>27.63790894188642</v>
       </c>
       <c r="AA582" t="inlineStr">
         <is>
@@ -80698,13 +80698,13 @@
         </is>
       </c>
       <c r="N583" t="n">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O583" t="n">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="R583" t="n">
-        <v>0.7565992348210768</v>
+        <v>0.7639448584601164</v>
       </c>
       <c r="AA583" t="inlineStr">
         <is>
@@ -81103,13 +81103,13 @@
         </is>
       </c>
       <c r="N586" t="n">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="O586" t="n">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="R586" t="n">
-        <v>0.9182029548799476</v>
+        <v>0.9292213903385069</v>
       </c>
       <c r="AA586" t="inlineStr">
         <is>
@@ -81778,13 +81778,13 @@
         </is>
       </c>
       <c r="N591" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="O591" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="R591" t="n">
-        <v>0.1542580964198312</v>
+        <v>0.1726221555174302</v>
       </c>
       <c r="AA591" t="inlineStr">
         <is>
@@ -81913,13 +81913,13 @@
         </is>
       </c>
       <c r="N592" t="n">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="O592" t="n">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="R592" t="n">
-        <v>2.824392289210718</v>
+        <v>2.842756348308317</v>
       </c>
       <c r="AA592" t="inlineStr">
         <is>
@@ -82048,13 +82048,13 @@
         </is>
       </c>
       <c r="N593" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O593" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="R593" t="n">
-        <v>0.2828065101030238</v>
+        <v>0.2901521337420634</v>
       </c>
       <c r="AA593" t="inlineStr">
         <is>
@@ -82183,13 +82183,13 @@
         </is>
       </c>
       <c r="N594" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="O594" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="R594" t="n">
-        <v>0.4848111601766123</v>
+        <v>0.4884839719961321</v>
       </c>
       <c r="AA594" t="inlineStr">
         <is>
@@ -82588,13 +82588,13 @@
         </is>
       </c>
       <c r="N597" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O597" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R597" t="n">
-        <v>0.02938249455615832</v>
+        <v>0.0367281181951979</v>
       </c>
       <c r="AA597" t="inlineStr">
         <is>
@@ -82993,13 +82993,13 @@
         </is>
       </c>
       <c r="N600" t="n">
-        <v>11286</v>
+        <v>11290</v>
       </c>
       <c r="O600" t="n">
-        <v>11286</v>
+        <v>11290</v>
       </c>
       <c r="R600" t="n">
-        <v>41.45135419510035</v>
+        <v>41.46604544237843</v>
       </c>
       <c r="AA600" t="inlineStr">
         <is>
@@ -83668,13 +83668,13 @@
         </is>
       </c>
       <c r="N605" t="n">
-        <v>3444</v>
+        <v>3452</v>
       </c>
       <c r="O605" t="n">
-        <v>3444</v>
+        <v>3452</v>
       </c>
       <c r="R605" t="n">
-        <v>12.64916390642616</v>
+        <v>12.67854640098232</v>
       </c>
       <c r="AA605" t="inlineStr">
         <is>
@@ -83803,13 +83803,13 @@
         </is>
       </c>
       <c r="N606" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O606" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R606" t="n">
-        <v>0.007345623639039581</v>
+        <v>0.00367281181951979</v>
       </c>
       <c r="AA606" t="inlineStr">
         <is>
@@ -85054,13 +85054,13 @@
         </is>
       </c>
       <c r="N615" t="n">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="O615" t="n">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="R615" t="n">
-        <v>7.066489940756076</v>
+        <v>7.062817128936556</v>
       </c>
       <c r="U615" t="inlineStr">
         <is>
@@ -85342,13 +85342,13 @@
         </is>
       </c>
       <c r="N617" t="n">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="O617" t="n">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="R617" t="n">
-        <v>1.483815975085995</v>
+        <v>1.527889716920233</v>
       </c>
       <c r="U617" t="inlineStr">
         <is>
@@ -85486,13 +85486,13 @@
         </is>
       </c>
       <c r="N618" t="n">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="O618" t="n">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="R618" t="n">
-        <v>0.8043457884748341</v>
+        <v>0.8337282830309923</v>
       </c>
       <c r="U618" t="inlineStr">
         <is>
@@ -85885,7 +85885,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>591953</v>
+        <v>592009</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-24 02:00:31 UTC
</commit_message>
<xml_diff>
--- a/countries/au/2026-2029.xlsx
+++ b/countries/au/2026-2029.xlsx
@@ -66594,13 +66594,13 @@
         </is>
       </c>
       <c r="N480" t="n">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="O480" t="n">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="R480" t="n">
-        <v>1.594000329671589</v>
+        <v>1.597673141491109</v>
       </c>
       <c r="U480" t="inlineStr">
         <is>
@@ -67962,13 +67962,13 @@
         </is>
       </c>
       <c r="N490" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O490" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="R490" t="n">
-        <v>0.4591014774399738</v>
+        <v>0.4554286656204539</v>
       </c>
       <c r="AA490" t="inlineStr">
         <is>
@@ -70703,13 +70703,13 @@
         </is>
       </c>
       <c r="N510" t="n">
-        <v>7519</v>
+        <v>7521</v>
       </c>
       <c r="O510" t="n">
-        <v>7519</v>
+        <v>7521</v>
       </c>
       <c r="R510" t="n">
-        <v>27.6158720709693</v>
+        <v>27.62321769460834</v>
       </c>
       <c r="AA510" t="inlineStr">
         <is>
@@ -71243,13 +71243,13 @@
         </is>
       </c>
       <c r="N514" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="O514" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="R514" t="n">
-        <v>1.120207604953536</v>
+        <v>1.123880416773056</v>
       </c>
       <c r="AA514" t="inlineStr">
         <is>
@@ -72188,13 +72188,13 @@
         </is>
       </c>
       <c r="N521" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O521" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R521" t="n">
-        <v>0.1542580964198312</v>
+        <v>0.157930908239351</v>
       </c>
       <c r="AA521" t="inlineStr">
         <is>
@@ -73808,13 +73808,13 @@
         </is>
       </c>
       <c r="N533" t="n">
-        <v>3614</v>
+        <v>3613</v>
       </c>
       <c r="O533" t="n">
-        <v>3614</v>
+        <v>3613</v>
       </c>
       <c r="R533" t="n">
-        <v>13.27354191574452</v>
+        <v>13.269869103925</v>
       </c>
       <c r="AA533" t="inlineStr">
         <is>
@@ -75626,13 +75626,13 @@
         </is>
       </c>
       <c r="N546" t="n">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="O546" t="n">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="R546" t="n">
-        <v>1.006350438548423</v>
+        <v>1.002677626728903</v>
       </c>
       <c r="U546" t="inlineStr">
         <is>
@@ -77957,13 +77957,13 @@
         </is>
       </c>
       <c r="N563" t="n">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="O563" t="n">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="R563" t="n">
-        <v>4.02540175419369</v>
+        <v>4.02907456601321</v>
       </c>
       <c r="AA563" t="inlineStr">
         <is>
@@ -78776,13 +78776,13 @@
         </is>
       </c>
       <c r="N569" t="n">
-        <v>71104</v>
+        <v>71105</v>
       </c>
       <c r="O569" t="n">
-        <v>71104</v>
+        <v>71105</v>
       </c>
       <c r="R569" t="n">
-        <v>261.1516116151352</v>
+        <v>261.1552844269547</v>
       </c>
       <c r="AA569" t="inlineStr">
         <is>
@@ -78911,13 +78911,13 @@
         </is>
       </c>
       <c r="N570" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O570" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R570" t="n">
-        <v>0.03305530637567811</v>
+        <v>0.02938249455615832</v>
       </c>
       <c r="AA570" t="inlineStr">
         <is>
@@ -80968,13 +80968,13 @@
         </is>
       </c>
       <c r="N585" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="O585" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="R585" t="n">
-        <v>0.7823089175577153</v>
+        <v>0.7859817293772351</v>
       </c>
       <c r="AA585" t="inlineStr">
         <is>
@@ -81103,13 +81103,13 @@
         </is>
       </c>
       <c r="N586" t="n">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O586" t="n">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="R586" t="n">
-        <v>0.9292213903385069</v>
+        <v>0.9255485785189871</v>
       </c>
       <c r="AA586" t="inlineStr">
         <is>
@@ -81238,13 +81238,13 @@
         </is>
       </c>
       <c r="N587" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O587" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="R587" t="n">
-        <v>0.209350273712628</v>
+        <v>0.2056774618931082</v>
       </c>
       <c r="AA587" t="inlineStr">
         <is>
@@ -81913,13 +81913,13 @@
         </is>
       </c>
       <c r="N592" t="n">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="O592" t="n">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="R592" t="n">
-        <v>2.842756348308317</v>
+        <v>2.853774783766877</v>
       </c>
       <c r="AA592" t="inlineStr">
         <is>
@@ -83668,13 +83668,13 @@
         </is>
       </c>
       <c r="N605" t="n">
-        <v>3452</v>
+        <v>3453</v>
       </c>
       <c r="O605" t="n">
-        <v>3452</v>
+        <v>3453</v>
       </c>
       <c r="R605" t="n">
-        <v>12.67854640098232</v>
+        <v>12.68221921280183</v>
       </c>
       <c r="AA605" t="inlineStr">
         <is>
@@ -84208,13 +84208,13 @@
         </is>
       </c>
       <c r="N609" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O609" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="R609" t="n">
-        <v>0.2938249455615832</v>
+        <v>0.3011705692006228</v>
       </c>
       <c r="AA609" t="inlineStr">
         <is>
@@ -85342,13 +85342,13 @@
         </is>
       </c>
       <c r="N617" t="n">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="O617" t="n">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="R617" t="n">
-        <v>1.527889716920233</v>
+        <v>1.538908152378792</v>
       </c>
       <c r="U617" t="inlineStr">
         <is>
@@ -85486,13 +85486,13 @@
         </is>
       </c>
       <c r="N618" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="O618" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="R618" t="n">
-        <v>0.8337282830309923</v>
+        <v>0.8374010948505122</v>
       </c>
       <c r="U618" t="inlineStr">
         <is>
@@ -85885,7 +85885,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>592009</v>
+        <v>592021</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-27 07:21:21 UTC
</commit_message>
<xml_diff>
--- a/countries/au/2026-2029.xlsx
+++ b/countries/au/2026-2029.xlsx
@@ -67962,13 +67962,13 @@
         </is>
       </c>
       <c r="N490" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O490" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="R490" t="n">
-        <v>0.4554286656204539</v>
+        <v>0.4517558538009342</v>
       </c>
       <c r="AA490" t="inlineStr">
         <is>
@@ -70703,13 +70703,13 @@
         </is>
       </c>
       <c r="N510" t="n">
-        <v>7521</v>
+        <v>7543</v>
       </c>
       <c r="O510" t="n">
-        <v>7521</v>
+        <v>7543</v>
       </c>
       <c r="R510" t="n">
-        <v>27.62321769460834</v>
+        <v>27.70401955463777</v>
       </c>
       <c r="AA510" t="inlineStr">
         <is>
@@ -75626,13 +75626,13 @@
         </is>
       </c>
       <c r="N546" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O546" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="R546" t="n">
-        <v>1.002677626728903</v>
+        <v>1.006350438548423</v>
       </c>
       <c r="U546" t="inlineStr">
         <is>
@@ -77957,13 +77957,13 @@
         </is>
       </c>
       <c r="N563" t="n">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="O563" t="n">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="R563" t="n">
-        <v>4.02907456601321</v>
+        <v>4.032747377832729</v>
       </c>
       <c r="AA563" t="inlineStr">
         <is>
@@ -78092,13 +78092,13 @@
         </is>
       </c>
       <c r="N564" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O564" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="R564" t="n">
-        <v>0.1689493436979103</v>
+        <v>0.1762949673369499</v>
       </c>
       <c r="AA564" t="inlineStr">
         <is>
@@ -78911,13 +78911,13 @@
         </is>
       </c>
       <c r="N570" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O570" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R570" t="n">
-        <v>0.02938249455615832</v>
+        <v>0.02203687091711874</v>
       </c>
       <c r="AA570" t="inlineStr">
         <is>
@@ -85342,13 +85342,13 @@
         </is>
       </c>
       <c r="N617" t="n">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="O617" t="n">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="R617" t="n">
-        <v>1.538908152378792</v>
+        <v>1.542580964198312</v>
       </c>
       <c r="U617" t="inlineStr">
         <is>
@@ -85885,7 +85885,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>592021</v>
+        <v>592045</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-29 03:23:46 UTC
</commit_message>
<xml_diff>
--- a/countries/au/2026-2029.xlsx
+++ b/countries/au/2026-2029.xlsx
@@ -70703,13 +70703,13 @@
         </is>
       </c>
       <c r="N510" t="n">
-        <v>7543</v>
+        <v>7544</v>
       </c>
       <c r="O510" t="n">
-        <v>7543</v>
+        <v>7544</v>
       </c>
       <c r="R510" t="n">
-        <v>27.70401955463777</v>
+        <v>27.70769236645729</v>
       </c>
       <c r="AA510" t="inlineStr">
         <is>
@@ -71243,13 +71243,13 @@
         </is>
       </c>
       <c r="N514" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O514" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="R514" t="n">
-        <v>1.123880416773056</v>
+        <v>1.127553228592576</v>
       </c>
       <c r="AA514" t="inlineStr">
         <is>
@@ -73133,13 +73133,13 @@
         </is>
       </c>
       <c r="N528" t="n">
-        <v>19126</v>
+        <v>19127</v>
       </c>
       <c r="O528" t="n">
-        <v>19126</v>
+        <v>19127</v>
       </c>
       <c r="R528" t="n">
-        <v>70.24619886013551</v>
+        <v>70.24987167195502</v>
       </c>
       <c r="AA528" t="inlineStr">
         <is>
@@ -75482,13 +75482,13 @@
         </is>
       </c>
       <c r="N545" t="n">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="O545" t="n">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="R545" t="n">
-        <v>1.832733097940375</v>
+        <v>1.836405909759895</v>
       </c>
       <c r="U545" t="inlineStr">
         <is>
@@ -76454,13 +76454,13 @@
         </is>
       </c>
       <c r="N552" t="n">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="O552" t="n">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="R552" t="n">
-        <v>1.531562528739753</v>
+        <v>1.527889716920233</v>
       </c>
       <c r="U552" t="inlineStr">
         <is>
@@ -76598,13 +76598,13 @@
         </is>
       </c>
       <c r="N553" t="n">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="O553" t="n">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="R553" t="n">
-        <v>1.766622485189019</v>
+        <v>1.762949673369499</v>
       </c>
       <c r="U553" t="inlineStr">
         <is>
@@ -76877,13 +76877,13 @@
         </is>
       </c>
       <c r="N555" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O555" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R555" t="n">
-        <v>0.00367281181951979</v>
+        <v>0</v>
       </c>
       <c r="AA555" t="inlineStr">
         <is>
@@ -77552,13 +77552,13 @@
         </is>
       </c>
       <c r="N560" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O560" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R560" t="n">
-        <v>0.209350273712628</v>
+        <v>0.2130230855321478</v>
       </c>
       <c r="AA560" t="inlineStr">
         <is>
@@ -77822,13 +77822,13 @@
         </is>
       </c>
       <c r="N562" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O562" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="R562" t="n">
-        <v>0.6023411384012456</v>
+        <v>0.5986683265817258</v>
       </c>
       <c r="AA562" t="inlineStr">
         <is>
@@ -77957,13 +77957,13 @@
         </is>
       </c>
       <c r="N563" t="n">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="O563" t="n">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="R563" t="n">
-        <v>4.036420189652249</v>
+        <v>4.040093001471769</v>
       </c>
       <c r="AA563" t="inlineStr">
         <is>
@@ -78776,13 +78776,13 @@
         </is>
       </c>
       <c r="N569" t="n">
-        <v>71107</v>
+        <v>71109</v>
       </c>
       <c r="O569" t="n">
-        <v>71107</v>
+        <v>71109</v>
       </c>
       <c r="R569" t="n">
-        <v>261.1626300505937</v>
+        <v>261.1699756742328</v>
       </c>
       <c r="AA569" t="inlineStr">
         <is>
@@ -80293,13 +80293,13 @@
         </is>
       </c>
       <c r="N580" t="n">
-        <v>3311</v>
+        <v>3312</v>
       </c>
       <c r="O580" t="n">
-        <v>3311</v>
+        <v>3312</v>
       </c>
       <c r="R580" t="n">
-        <v>12.16067993443002</v>
+        <v>12.16435274624954</v>
       </c>
       <c r="AA580" t="inlineStr">
         <is>
@@ -80968,13 +80968,13 @@
         </is>
       </c>
       <c r="N585" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O585" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="R585" t="n">
-        <v>0.7933273530162747</v>
+        <v>0.7970001648357945</v>
       </c>
       <c r="AA585" t="inlineStr">
         <is>
@@ -81103,13 +81103,13 @@
         </is>
       </c>
       <c r="N586" t="n">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O586" t="n">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="R586" t="n">
-        <v>0.9292213903385069</v>
+        <v>0.9255485785189871</v>
       </c>
       <c r="AA586" t="inlineStr">
         <is>
@@ -81778,13 +81778,13 @@
         </is>
       </c>
       <c r="N591" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O591" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="R591" t="n">
-        <v>0.1726221555174302</v>
+        <v>0.1762949673369499</v>
       </c>
       <c r="AA591" t="inlineStr">
         <is>
@@ -81913,13 +81913,13 @@
         </is>
       </c>
       <c r="N592" t="n">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="O592" t="n">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="R592" t="n">
-        <v>2.857447595586397</v>
+        <v>2.861120407405917</v>
       </c>
       <c r="AA592" t="inlineStr">
         <is>
@@ -82183,13 +82183,13 @@
         </is>
       </c>
       <c r="N594" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O594" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="R594" t="n">
-        <v>0.4884839719961321</v>
+        <v>0.4921567838156519</v>
       </c>
       <c r="AA594" t="inlineStr">
         <is>
@@ -83668,13 +83668,13 @@
         </is>
       </c>
       <c r="N605" t="n">
-        <v>3454</v>
+        <v>3453</v>
       </c>
       <c r="O605" t="n">
-        <v>3454</v>
+        <v>3453</v>
       </c>
       <c r="R605" t="n">
-        <v>12.68589202462135</v>
+        <v>12.68221921280183</v>
       </c>
       <c r="AA605" t="inlineStr">
         <is>
@@ -84208,13 +84208,13 @@
         </is>
       </c>
       <c r="N609" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O609" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="R609" t="n">
-        <v>0.3048433810201426</v>
+        <v>0.3085161928396624</v>
       </c>
       <c r="AA609" t="inlineStr">
         <is>
@@ -85342,13 +85342,13 @@
         </is>
       </c>
       <c r="N617" t="n">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="O617" t="n">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="R617" t="n">
-        <v>1.542580964198312</v>
+        <v>1.553599399656871</v>
       </c>
       <c r="U617" t="inlineStr">
         <is>
@@ -85486,13 +85486,13 @@
         </is>
       </c>
       <c r="N618" t="n">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="O618" t="n">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="R618" t="n">
-        <v>0.841073906670032</v>
+        <v>0.8484195303090715</v>
       </c>
       <c r="U618" t="inlineStr">
         <is>
@@ -95745,7 +95745,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>663199</v>
+        <v>663212</v>
       </c>
     </row>
     <row r="16">

</xml_diff>